<commit_message>
Daily slate 2026-06-08 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-06.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-06.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="E2" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F2" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="G2" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E3" t="n">
         <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G3" t="n">
-        <v>53.8</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G4" t="n">
-        <v>28.8</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="E5" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F5" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G5" t="n">
-        <v>48.8</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E6" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F6" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G6" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
       </c>
       <c r="G7" t="n">
-        <v>69.2</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -674,13 +674,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>977</v>
+        <v>1093</v>
       </c>
       <c r="E11" t="n">
-        <v>540</v>
+        <v>608</v>
       </c>
       <c r="F11" t="n">
-        <v>437</v>
+        <v>485</v>
       </c>
       <c r="G11" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="E12" t="n">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="F12" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G12" t="n">
-        <v>69.90000000000001</v>
+        <v>69.09999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F13" t="n">
         <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>41.7</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>312</v>
+        <v>343</v>
       </c>
       <c r="E14" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F14" t="n">
-        <v>235</v>
+        <v>259</v>
       </c>
       <c r="G14" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>413</v>
+        <v>440</v>
       </c>
       <c r="E15" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F15" t="n">
-        <v>331</v>
+        <v>354</v>
       </c>
       <c r="G15" t="n">
-        <v>19.9</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="E16" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F16" t="n">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="G16" t="n">
-        <v>19.2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3809</v>
+        <v>4320</v>
       </c>
       <c r="E17" t="n">
-        <v>753</v>
+        <v>884</v>
       </c>
       <c r="F17" t="n">
-        <v>3056</v>
+        <v>3436</v>
       </c>
       <c r="G17" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
     </row>
   </sheetData>
@@ -1528,64 +1528,64 @@
         <v>126</v>
       </c>
       <c r="D7" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
       <c r="E7" t="n">
-        <v>977</v>
+        <v>1093</v>
       </c>
       <c r="F7" t="n">
-        <v>69.90000000000001</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="H7" t="n">
-        <v>41.7</v>
+        <v>42.9</v>
       </c>
       <c r="I7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J7" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
       <c r="K7" t="n">
-        <v>312</v>
+        <v>343</v>
       </c>
       <c r="L7" t="n">
-        <v>19.9</v>
+        <v>19.5</v>
       </c>
       <c r="M7" t="n">
-        <v>413</v>
+        <v>440</v>
       </c>
       <c r="N7" t="n">
-        <v>19.2</v>
+        <v>19</v>
       </c>
       <c r="O7" t="n">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="P7" t="n">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>3809</v>
+        <v>4320</v>
       </c>
       <c r="R7" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="S7" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="T7" t="n">
-        <v>28.8</v>
+        <v>32.1</v>
       </c>
       <c r="U7" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="V7" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="W7" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="X7" t="n">
         <v>39.5</v>
@@ -1594,28 +1594,28 @@
         <v>349</v>
       </c>
       <c r="Z7" t="n">
-        <v>53.8</v>
+        <v>53</v>
       </c>
       <c r="AA7" t="n">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="AB7" t="n">
-        <v>48.8</v>
+        <v>48.9</v>
       </c>
       <c r="AC7" t="n">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="AD7" t="n">
-        <v>69.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AE7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AF7" t="n">
         <v>0</v>
       </c>
       <c r="AG7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>